<commit_message>
added to missing cells
</commit_message>
<xml_diff>
--- a/Data/Initial_Database.xlsx
+++ b/Data/Initial_Database.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jerry\Documents\GitHub\Methane_Prediction\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhang\Documents\GitHub\Methane_Prediction\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09EA9331-F771-4BC2-8FEB-B37C34AAF0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00E3A4AD-3315-411D-B87A-CE0CF7D13412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
@@ -244,17 +244,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -314,7 +314,7 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -502,7 +502,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="58" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -569,7 +569,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -848,24 +848,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T251"/>
-  <sheetFormatPr defaultRowHeight="20.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="20.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="21.90625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="16.7265625" style="14" customWidth="1"/>
-    <col min="4" max="6" width="11.7265625" style="14" customWidth="1"/>
-    <col min="7" max="7" width="15.7265625" style="14" customWidth="1"/>
-    <col min="8" max="8" width="19.7265625" style="14" customWidth="1"/>
-    <col min="9" max="9" width="18.6328125" style="14" customWidth="1"/>
-    <col min="10" max="10" width="11.7265625" style="14" customWidth="1"/>
-    <col min="11" max="11" width="12.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.73046875" style="14" customWidth="1"/>
+    <col min="2" max="2" width="21.9296875" style="14" customWidth="1"/>
+    <col min="3" max="3" width="16.73046875" style="14" customWidth="1"/>
+    <col min="4" max="6" width="11.73046875" style="14" customWidth="1"/>
+    <col min="7" max="7" width="15.73046875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="19.73046875" style="14" customWidth="1"/>
+    <col min="9" max="9" width="18.59765625" style="14" customWidth="1"/>
+    <col min="10" max="10" width="11.73046875" style="14" customWidth="1"/>
+    <col min="11" max="11" width="12.9296875" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="16" width="9" style="1"/>
-    <col min="17" max="17" width="9.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="13.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.06640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="13.59765625" style="1" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="9" customFormat="1" ht="80" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" s="9" customFormat="1" ht="79.900000000000006">
       <c r="A1" s="12" t="s">
         <v>2</v>
       </c>
@@ -907,7 +907,7 @@
       <c r="S1" s="8"/>
       <c r="T1" s="8"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20">
       <c r="A2" s="13">
         <v>1</v>
       </c>
@@ -930,7 +930,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20">
       <c r="A3" s="13">
         <v>1</v>
       </c>
@@ -953,7 +953,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:20">
       <c r="A4" s="13">
         <v>1</v>
       </c>
@@ -976,7 +976,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:20">
       <c r="A5" s="13">
         <v>1</v>
       </c>
@@ -999,7 +999,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:20">
       <c r="A6" s="13">
         <v>1</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:20">
       <c r="A7" s="13">
         <v>1</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:20">
       <c r="A8" s="13">
         <v>1</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:20">
       <c r="A9" s="13">
         <v>1</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:20">
       <c r="A10" s="13">
         <v>1</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:20">
       <c r="A11" s="13">
         <v>1</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:20">
       <c r="A12" s="13">
         <v>1</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:20">
       <c r="A13" s="13">
         <v>1</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:20">
       <c r="A14" s="13">
         <v>1</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:20">
       <c r="A15" s="13">
         <v>1</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:20">
       <c r="A16" s="13">
         <v>1</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7">
       <c r="A17" s="13">
         <v>1</v>
       </c>
@@ -1275,7 +1275,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7">
       <c r="A18" s="13">
         <v>1</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7">
       <c r="A19" s="13">
         <v>1</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7">
       <c r="A20" s="13">
         <v>1</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7">
       <c r="A21" s="13">
         <v>1</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7">
       <c r="A22" s="16">
         <v>1</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7">
       <c r="A23" s="18">
         <v>2</v>
       </c>
@@ -1413,7 +1413,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7">
       <c r="A24" s="13">
         <v>2</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7">
       <c r="A25" s="13">
         <v>2</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7">
       <c r="A26" s="13">
         <v>2</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7">
       <c r="A27" s="13">
         <v>2</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7">
       <c r="A28" s="13">
         <v>2</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7">
       <c r="A29" s="13">
         <v>2</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7">
       <c r="A30" s="13">
         <v>2</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7">
       <c r="A31" s="13">
         <v>2</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7">
       <c r="A32" s="13">
         <v>2</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7">
       <c r="A33" s="13">
         <v>2</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7">
       <c r="A34" s="13">
         <v>2</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7">
       <c r="A35" s="13">
         <v>2</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7">
       <c r="A36" s="13">
         <v>2</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7">
       <c r="A37" s="13">
         <v>2</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7">
       <c r="A38" s="13">
         <v>2</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7">
       <c r="A39" s="13">
         <v>2</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7">
       <c r="A40" s="13">
         <v>2</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7">
       <c r="A41" s="13">
         <v>2</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7">
       <c r="A42" s="13">
         <v>2</v>
       </c>
@@ -1850,7 +1850,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7">
       <c r="A43" s="13">
         <v>2</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7">
       <c r="A44" s="16">
         <v>2</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7">
       <c r="A45" s="18">
         <v>3</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7">
       <c r="A46" s="13">
         <v>3</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7">
       <c r="A47" s="13">
         <v>3</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7">
       <c r="A48" s="13">
         <v>3</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:19">
       <c r="A49" s="13">
         <v>3</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:19">
       <c r="A50" s="13">
         <v>3</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:19">
       <c r="A51" s="13">
         <v>3</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:19">
       <c r="A52" s="13">
         <v>3</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:19">
       <c r="A53" s="13">
         <v>3</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:19">
       <c r="A54" s="13">
         <v>3</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:19">
       <c r="A55" s="13">
         <v>3</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:19">
       <c r="A56" s="13">
         <v>3</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:19">
       <c r="A57" s="13">
         <v>3</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:19">
       <c r="A58" s="13">
         <v>3</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:19">
       <c r="A59" s="13">
         <v>3</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:19">
       <c r="A60" s="13">
         <v>3</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="61" spans="1:19" ht="20.65" thickBot="1">
       <c r="A61" s="21">
         <v>3</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="22" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="62" spans="1:19" ht="21.4" thickBot="1">
       <c r="A62" s="23">
         <v>4</v>
       </c>
@@ -2322,7 +2322,7 @@
       <c r="R62" s="3"/>
       <c r="S62" s="3"/>
     </row>
-    <row r="63" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="63" spans="1:19" ht="20.65" thickBot="1">
       <c r="A63" s="27">
         <v>4</v>
       </c>
@@ -2346,12 +2346,15 @@
       </c>
       <c r="H63" s="26">
         <v>1351.6258170000001</v>
+      </c>
+      <c r="I63" s="14">
+        <v>212</v>
       </c>
       <c r="Q63" s="2"/>
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
     </row>
-    <row r="64" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="64" spans="1:19" ht="20.65" thickBot="1">
       <c r="A64" s="27">
         <v>4</v>
       </c>
@@ -2375,12 +2378,15 @@
       </c>
       <c r="H64" s="26">
         <v>2649.1869919999999</v>
+      </c>
+      <c r="I64" s="14">
+        <v>212</v>
       </c>
       <c r="Q64" s="2"/>
       <c r="R64" s="2"/>
       <c r="S64" s="2"/>
     </row>
-    <row r="65" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="65" spans="1:19" ht="20.65" thickBot="1">
       <c r="A65" s="27">
         <v>4</v>
       </c>
@@ -2404,12 +2410,15 @@
       </c>
       <c r="H65" s="26">
         <v>3514.2276430000002</v>
+      </c>
+      <c r="I65" s="14">
+        <v>212</v>
       </c>
       <c r="Q65" s="2"/>
       <c r="R65" s="2"/>
       <c r="S65" s="2"/>
     </row>
-    <row r="66" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="66" spans="1:19" ht="20.65" thickBot="1">
       <c r="A66" s="27">
         <v>4</v>
       </c>
@@ -2433,12 +2442,15 @@
       </c>
       <c r="H66" s="26">
         <v>6325.6097559999998</v>
+      </c>
+      <c r="I66" s="14">
+        <v>212</v>
       </c>
       <c r="Q66" s="2"/>
       <c r="R66" s="2"/>
       <c r="S66" s="2"/>
     </row>
-    <row r="67" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="67" spans="1:19" ht="20.65" thickBot="1">
       <c r="A67" s="27">
         <v>4</v>
       </c>
@@ -2462,12 +2474,15 @@
       </c>
       <c r="H67" s="26">
         <v>4000.8130080000001</v>
+      </c>
+      <c r="I67" s="14">
+        <v>212</v>
       </c>
       <c r="Q67" s="2"/>
       <c r="R67" s="2"/>
       <c r="S67" s="2"/>
     </row>
-    <row r="68" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="68" spans="1:19" ht="20.65" thickBot="1">
       <c r="A68" s="27">
         <v>4</v>
       </c>
@@ -2491,12 +2506,15 @@
       </c>
       <c r="H68" s="26">
         <v>4919.9186989999998</v>
+      </c>
+      <c r="I68" s="14">
+        <v>212</v>
       </c>
       <c r="Q68" s="2"/>
       <c r="R68" s="2"/>
       <c r="S68" s="2"/>
     </row>
-    <row r="69" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="69" spans="1:19" ht="20.65" thickBot="1">
       <c r="A69" s="27">
         <v>4</v>
       </c>
@@ -2520,12 +2538,15 @@
       </c>
       <c r="H69" s="26">
         <v>4217.0731699999997</v>
+      </c>
+      <c r="I69" s="14">
+        <v>212</v>
       </c>
       <c r="Q69" s="2"/>
       <c r="R69" s="2"/>
       <c r="S69" s="2"/>
     </row>
-    <row r="70" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="70" spans="1:19" ht="20.65" thickBot="1">
       <c r="A70" s="27">
         <v>4</v>
       </c>
@@ -2549,12 +2570,15 @@
       </c>
       <c r="H70" s="26">
         <v>4487.3983740000003</v>
+      </c>
+      <c r="I70" s="14">
+        <v>212</v>
       </c>
       <c r="Q70" s="2"/>
       <c r="R70" s="2"/>
       <c r="S70" s="2"/>
     </row>
-    <row r="71" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="71" spans="1:19" ht="20.65" thickBot="1">
       <c r="A71" s="27">
         <v>4</v>
       </c>
@@ -2578,12 +2602,15 @@
       </c>
       <c r="H71" s="26">
         <v>5839.0243899999996</v>
+      </c>
+      <c r="I71" s="14">
+        <v>212</v>
       </c>
       <c r="Q71" s="2"/>
       <c r="R71" s="2"/>
       <c r="S71" s="2"/>
     </row>
-    <row r="72" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="72" spans="1:19" ht="20.65" thickBot="1">
       <c r="A72" s="27">
         <v>4</v>
       </c>
@@ -2607,12 +2634,15 @@
       </c>
       <c r="H72" s="26">
         <v>3946.7479680000001</v>
+      </c>
+      <c r="I72" s="14">
+        <v>212</v>
       </c>
       <c r="Q72" s="2"/>
       <c r="R72" s="2"/>
       <c r="S72" s="2"/>
     </row>
-    <row r="73" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="73" spans="1:19" ht="20.65" thickBot="1">
       <c r="A73" s="27">
         <v>4</v>
       </c>
@@ -2636,12 +2666,15 @@
       </c>
       <c r="H73" s="26">
         <v>3297.9674799999998</v>
+      </c>
+      <c r="I73" s="14">
+        <v>212</v>
       </c>
       <c r="Q73" s="2"/>
       <c r="R73" s="2"/>
       <c r="S73" s="2"/>
     </row>
-    <row r="74" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="74" spans="1:19" ht="20.65" thickBot="1">
       <c r="A74" s="27">
         <v>4</v>
       </c>
@@ -2665,12 +2698,15 @@
       </c>
       <c r="H74" s="26">
         <v>3406.097561</v>
+      </c>
+      <c r="I74" s="14">
+        <v>212</v>
       </c>
       <c r="Q74" s="2"/>
       <c r="R74" s="2"/>
       <c r="S74" s="2"/>
     </row>
-    <row r="75" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="75" spans="1:19" ht="20.65" thickBot="1">
       <c r="A75" s="27">
         <v>4</v>
       </c>
@@ -2694,12 +2730,15 @@
       </c>
       <c r="H75" s="26">
         <v>2973.5772360000001</v>
+      </c>
+      <c r="I75" s="14">
+        <v>212</v>
       </c>
       <c r="Q75" s="2"/>
       <c r="R75" s="2"/>
       <c r="S75" s="2"/>
     </row>
-    <row r="76" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="76" spans="1:19" ht="20.65" thickBot="1">
       <c r="A76" s="27">
         <v>4</v>
       </c>
@@ -2723,12 +2762,15 @@
       </c>
       <c r="H76" s="26">
         <v>3189.837399</v>
+      </c>
+      <c r="I76" s="14">
+        <v>212</v>
       </c>
       <c r="Q76" s="2"/>
       <c r="R76" s="2"/>
       <c r="S76" s="2"/>
     </row>
-    <row r="77" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="77" spans="1:19" ht="20.65" thickBot="1">
       <c r="A77" s="27">
         <v>4</v>
       </c>
@@ -2752,12 +2794,15 @@
       </c>
       <c r="H77" s="26">
         <v>3243.902439</v>
+      </c>
+      <c r="I77" s="14">
+        <v>212</v>
       </c>
       <c r="Q77" s="2"/>
       <c r="R77" s="2"/>
       <c r="S77" s="2"/>
     </row>
-    <row r="78" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="78" spans="1:19" ht="20.65" thickBot="1">
       <c r="A78" s="27">
         <v>4</v>
       </c>
@@ -2781,12 +2826,15 @@
       </c>
       <c r="H78" s="26">
         <v>1838.211382</v>
+      </c>
+      <c r="I78" s="14">
+        <v>212</v>
       </c>
       <c r="Q78" s="2"/>
       <c r="R78" s="2"/>
       <c r="S78" s="2"/>
     </row>
-    <row r="79" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="79" spans="1:19" ht="20.65" thickBot="1">
       <c r="A79" s="27">
         <v>4</v>
       </c>
@@ -2810,12 +2858,15 @@
       </c>
       <c r="H79" s="26">
         <v>2054.4715449999999</v>
+      </c>
+      <c r="I79" s="14">
+        <v>212</v>
       </c>
       <c r="Q79" s="2"/>
       <c r="R79" s="2"/>
       <c r="S79" s="2"/>
     </row>
-    <row r="80" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="80" spans="1:19" ht="20.65" thickBot="1">
       <c r="A80" s="27">
         <v>4</v>
       </c>
@@ -2839,12 +2890,15 @@
       </c>
       <c r="H80" s="26">
         <v>2108.5365860000002</v>
+      </c>
+      <c r="I80" s="14">
+        <v>212</v>
       </c>
       <c r="Q80" s="2"/>
       <c r="R80" s="2"/>
       <c r="S80" s="2"/>
     </row>
-    <row r="81" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="81" spans="1:19" ht="20.65" thickBot="1">
       <c r="A81" s="27">
         <v>4</v>
       </c>
@@ -2868,12 +2922,15 @@
       </c>
       <c r="H81" s="26">
         <v>1838.211382</v>
+      </c>
+      <c r="I81" s="14">
+        <v>212</v>
       </c>
       <c r="Q81" s="2"/>
       <c r="R81" s="2"/>
       <c r="S81" s="2"/>
     </row>
-    <row r="82" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="82" spans="1:19" ht="20.65" thickBot="1">
       <c r="A82" s="27">
         <v>4</v>
       </c>
@@ -2897,12 +2954,15 @@
       </c>
       <c r="H82" s="26">
         <v>865.04065000000003</v>
+      </c>
+      <c r="I82" s="14">
+        <v>212</v>
       </c>
       <c r="Q82" s="2"/>
       <c r="R82" s="2"/>
       <c r="S82" s="2"/>
     </row>
-    <row r="83" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="83" spans="1:19" ht="20.65" thickBot="1">
       <c r="A83" s="27">
         <v>4</v>
       </c>
@@ -2926,12 +2986,15 @@
       </c>
       <c r="H83" s="26">
         <v>756.91057000000001</v>
+      </c>
+      <c r="I83" s="14">
+        <v>212</v>
       </c>
       <c r="Q83" s="2"/>
       <c r="R83" s="2"/>
       <c r="S83" s="2"/>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:19">
       <c r="A84" s="28">
         <v>4</v>
       </c>
@@ -2955,12 +3018,15 @@
       </c>
       <c r="H84" s="26">
         <v>432.52032500000001</v>
+      </c>
+      <c r="I84" s="14">
+        <v>212</v>
       </c>
       <c r="Q84" s="2"/>
       <c r="R84" s="2"/>
       <c r="S84" s="2"/>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:19">
       <c r="A85" s="29">
         <v>5</v>
       </c>
@@ -2992,7 +3058,7 @@
       <c r="R85" s="2"/>
       <c r="S85" s="2"/>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:19">
       <c r="A86" s="27">
         <v>5</v>
       </c>
@@ -3016,12 +3082,15 @@
       </c>
       <c r="H86" s="26">
         <v>68.578767999999997</v>
+      </c>
+      <c r="I86" s="14">
+        <v>153</v>
       </c>
       <c r="Q86" s="2"/>
       <c r="R86" s="2"/>
       <c r="S86" s="2"/>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:19">
       <c r="A87" s="27">
         <v>5</v>
       </c>
@@ -3045,12 +3114,15 @@
       </c>
       <c r="H87" s="26">
         <v>380.73702700000001</v>
+      </c>
+      <c r="I87" s="14">
+        <v>153</v>
       </c>
       <c r="Q87" s="2"/>
       <c r="R87" s="2"/>
       <c r="S87" s="2"/>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:19">
       <c r="A88" s="27">
         <v>5</v>
       </c>
@@ -3074,12 +3146,15 @@
       </c>
       <c r="H88" s="26">
         <v>982.22139700000002</v>
+      </c>
+      <c r="I88" s="14">
+        <v>153</v>
       </c>
       <c r="Q88" s="2"/>
       <c r="R88" s="2"/>
       <c r="S88" s="2"/>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:19">
       <c r="A89" s="27">
         <v>5</v>
       </c>
@@ -3103,12 +3178,15 @@
       </c>
       <c r="H89" s="26">
         <v>1227.4748790000001</v>
+      </c>
+      <c r="I89" s="14">
+        <v>153</v>
       </c>
       <c r="Q89" s="2"/>
       <c r="R89" s="2"/>
       <c r="S89" s="2"/>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:19">
       <c r="A90" s="27">
         <v>5</v>
       </c>
@@ -3132,12 +3210,15 @@
       </c>
       <c r="H90" s="26">
         <v>3184.727742</v>
+      </c>
+      <c r="I90" s="14">
+        <v>153</v>
       </c>
       <c r="Q90" s="2"/>
       <c r="R90" s="2"/>
       <c r="S90" s="2"/>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:19">
       <c r="A91" s="27">
         <v>5</v>
       </c>
@@ -3161,12 +3242,15 @@
       </c>
       <c r="H91" s="26">
         <v>2562.469411</v>
+      </c>
+      <c r="I91" s="14">
+        <v>153</v>
       </c>
       <c r="Q91" s="2"/>
       <c r="R91" s="2"/>
       <c r="S91" s="2"/>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:19">
       <c r="A92" s="27">
         <v>5</v>
       </c>
@@ -3190,12 +3274,15 @@
       </c>
       <c r="H92" s="26">
         <v>3029.595378</v>
+      </c>
+      <c r="I92" s="14">
+        <v>153</v>
       </c>
       <c r="Q92" s="2"/>
       <c r="R92" s="2"/>
       <c r="S92" s="2"/>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:19">
       <c r="A93" s="27">
         <v>5</v>
       </c>
@@ -3219,12 +3306,15 @@
       </c>
       <c r="H93" s="26">
         <v>3052.454968</v>
+      </c>
+      <c r="I93" s="14">
+        <v>153</v>
       </c>
       <c r="Q93" s="2"/>
       <c r="R93" s="2"/>
       <c r="S93" s="2"/>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:19">
       <c r="A94" s="27">
         <v>5</v>
       </c>
@@ -3248,12 +3338,15 @@
       </c>
       <c r="H94" s="26">
         <v>2874.9295360000001</v>
+      </c>
+      <c r="I94" s="14">
+        <v>153</v>
       </c>
       <c r="Q94" s="2"/>
       <c r="R94" s="2"/>
       <c r="S94" s="2"/>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:19">
       <c r="A95" s="27">
         <v>5</v>
       </c>
@@ -3277,12 +3370,15 @@
       </c>
       <c r="H95" s="26">
         <v>2808.4363979999998</v>
+      </c>
+      <c r="I95" s="14">
+        <v>153</v>
       </c>
       <c r="Q95" s="2"/>
       <c r="R95" s="2"/>
       <c r="S95" s="2"/>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:19">
       <c r="A96" s="27">
         <v>5</v>
       </c>
@@ -3306,12 +3402,15 @@
       </c>
       <c r="H96" s="26">
         <v>3386.4848870000001</v>
+      </c>
+      <c r="I96" s="14">
+        <v>153</v>
       </c>
       <c r="Q96" s="2"/>
       <c r="R96" s="2"/>
       <c r="S96" s="2"/>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:19">
       <c r="A97" s="27">
         <v>5</v>
       </c>
@@ -3335,12 +3434,15 @@
       </c>
       <c r="H97" s="26">
         <v>3520.3767670000002</v>
+      </c>
+      <c r="I97" s="14">
+        <v>153</v>
       </c>
       <c r="Q97" s="2"/>
       <c r="R97" s="2"/>
       <c r="S97" s="2"/>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:19">
       <c r="A98" s="27">
         <v>5</v>
       </c>
@@ -3364,12 +3466,15 @@
       </c>
       <c r="H98" s="26">
         <v>4365.3308569999999</v>
+      </c>
+      <c r="I98" s="14">
+        <v>153</v>
       </c>
       <c r="Q98" s="2"/>
       <c r="R98" s="2"/>
       <c r="S98" s="2"/>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:19">
       <c r="A99" s="27">
         <v>5</v>
       </c>
@@ -3393,12 +3498,15 @@
       </c>
       <c r="H99" s="26">
         <v>5188.5779430000002</v>
+      </c>
+      <c r="I99" s="14">
+        <v>153</v>
       </c>
       <c r="Q99" s="2"/>
       <c r="R99" s="2"/>
       <c r="S99" s="2"/>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:19">
       <c r="A100" s="27">
         <v>5</v>
       </c>
@@ -3422,12 +3530,15 @@
       </c>
       <c r="H100" s="26">
         <v>3010.3856390000001</v>
+      </c>
+      <c r="I100" s="14">
+        <v>153</v>
       </c>
       <c r="Q100" s="2"/>
       <c r="R100" s="2"/>
       <c r="S100" s="2"/>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:19">
       <c r="A101" s="27">
         <v>5</v>
       </c>
@@ -3451,12 +3562,15 @@
       </c>
       <c r="H101" s="26">
         <v>2833.6560399999998</v>
+      </c>
+      <c r="I101" s="14">
+        <v>153</v>
       </c>
       <c r="Q101" s="2"/>
       <c r="R101" s="2"/>
       <c r="S101" s="2"/>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:19">
       <c r="A102" s="27">
         <v>5</v>
       </c>
@@ -3480,12 +3594,15 @@
       </c>
       <c r="H102" s="26">
         <v>1367.8431860000001</v>
+      </c>
+      <c r="I102" s="14">
+        <v>153</v>
       </c>
       <c r="Q102" s="2"/>
       <c r="R102" s="2"/>
       <c r="S102" s="2"/>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:19">
       <c r="A103" s="27">
         <v>5</v>
       </c>
@@ -3509,12 +3626,15 @@
       </c>
       <c r="H103" s="26">
         <v>2191.419582</v>
+      </c>
+      <c r="I103" s="14">
+        <v>153</v>
       </c>
       <c r="Q103" s="2"/>
       <c r="R103" s="2"/>
       <c r="S103" s="2"/>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:19">
       <c r="A104" s="27">
         <v>5</v>
       </c>
@@ -3538,12 +3658,15 @@
       </c>
       <c r="H104" s="26">
         <v>1525.829567</v>
+      </c>
+      <c r="I104" s="14">
+        <v>153</v>
       </c>
       <c r="Q104" s="2"/>
       <c r="R104" s="2"/>
       <c r="S104" s="2"/>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:19">
       <c r="A105" s="27">
         <v>5</v>
       </c>
@@ -3567,12 +3690,15 @@
       </c>
       <c r="H105" s="26">
         <v>82.080470000000005</v>
+      </c>
+      <c r="I105" s="14">
+        <v>153</v>
       </c>
       <c r="Q105" s="2"/>
       <c r="R105" s="2"/>
       <c r="S105" s="2"/>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:19">
       <c r="A106" s="27">
         <v>5</v>
       </c>
@@ -3596,12 +3722,15 @@
       </c>
       <c r="H106" s="26">
         <v>950.11369000000002</v>
+      </c>
+      <c r="I106" s="14">
+        <v>153</v>
       </c>
       <c r="Q106" s="2"/>
       <c r="R106" s="2"/>
       <c r="S106" s="2"/>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:19">
       <c r="A107" s="27">
         <v>5</v>
       </c>
@@ -3625,12 +3754,15 @@
       </c>
       <c r="H107" s="26">
         <v>506.80779899999999</v>
+      </c>
+      <c r="I107" s="14">
+        <v>153</v>
       </c>
       <c r="Q107" s="2"/>
       <c r="R107" s="2"/>
       <c r="S107" s="2"/>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:19">
       <c r="A108" s="27">
         <v>5</v>
       </c>
@@ -3654,12 +3786,15 @@
       </c>
       <c r="H108" s="26">
         <v>485.04590899999999</v>
+      </c>
+      <c r="I108" s="14">
+        <v>153</v>
       </c>
       <c r="Q108" s="2"/>
       <c r="R108" s="2"/>
       <c r="S108" s="2"/>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:19">
       <c r="A109" s="27">
         <v>5</v>
       </c>
@@ -3683,12 +3818,15 @@
       </c>
       <c r="H109" s="26">
         <v>463.14680700000002</v>
+      </c>
+      <c r="I109" s="14">
+        <v>153</v>
       </c>
       <c r="Q109" s="2"/>
       <c r="R109" s="2"/>
       <c r="S109" s="2"/>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:19">
       <c r="A110" s="27">
         <v>5</v>
       </c>
@@ -3712,12 +3850,15 @@
       </c>
       <c r="H110" s="26">
         <v>2019.4924169999999</v>
+      </c>
+      <c r="I110" s="14">
+        <v>153</v>
       </c>
       <c r="Q110" s="2"/>
       <c r="R110" s="2"/>
       <c r="S110" s="2"/>
     </row>
-    <row r="111" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="111" spans="1:19" ht="20.65" thickBot="1">
       <c r="A111" s="30">
         <v>5</v>
       </c>
@@ -3741,13 +3882,16 @@
       </c>
       <c r="H111" s="26">
         <v>19.539048999999999</v>
+      </c>
+      <c r="I111" s="14">
+        <v>153</v>
       </c>
       <c r="L111" s="4"/>
       <c r="Q111" s="2"/>
       <c r="R111" s="2"/>
       <c r="S111" s="2"/>
     </row>
-    <row r="112" spans="1:19" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="112" spans="1:19" ht="20.65" thickBot="1">
       <c r="A112" s="31">
         <v>6</v>
       </c>
@@ -3780,7 +3924,7 @@
       <c r="R112" s="2"/>
       <c r="S112" s="2"/>
     </row>
-    <row r="113" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="113" spans="1:12" ht="20.65" thickBot="1">
       <c r="A113" s="34">
         <v>6</v>
       </c>
@@ -3805,10 +3949,12 @@
       <c r="H113" s="33">
         <v>334.81649609999999</v>
       </c>
-      <c r="I113" s="33"/>
+      <c r="I113" s="14">
+        <v>401</v>
+      </c>
       <c r="L113" s="5"/>
     </row>
-    <row r="114" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="114" spans="1:12" ht="20.65" thickBot="1">
       <c r="A114" s="34">
         <v>6</v>
       </c>
@@ -3833,10 +3979,12 @@
       <c r="H114" s="33">
         <v>2696.8962729999998</v>
       </c>
-      <c r="I114" s="33"/>
+      <c r="I114" s="14">
+        <v>401</v>
+      </c>
       <c r="L114" s="5"/>
     </row>
-    <row r="115" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="115" spans="1:12" ht="20.65" thickBot="1">
       <c r="A115" s="34">
         <v>6</v>
       </c>
@@ -3861,10 +4009,12 @@
       <c r="H115" s="33">
         <v>1966.0119950000001</v>
       </c>
-      <c r="I115" s="33"/>
+      <c r="I115" s="14">
+        <v>401</v>
+      </c>
       <c r="L115" s="5"/>
     </row>
-    <row r="116" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="116" spans="1:12" ht="20.65" thickBot="1">
       <c r="A116" s="34">
         <v>6</v>
       </c>
@@ -3889,10 +4039,12 @@
       <c r="H116" s="33">
         <v>2896.9985809999998</v>
       </c>
-      <c r="I116" s="33"/>
+      <c r="I116" s="14">
+        <v>401</v>
+      </c>
       <c r="L116" s="5"/>
     </row>
-    <row r="117" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="117" spans="1:12" ht="20.65" thickBot="1">
       <c r="A117" s="34">
         <v>6</v>
       </c>
@@ -3917,10 +4069,12 @@
       <c r="H117" s="33">
         <v>1733.8620080000001</v>
       </c>
-      <c r="I117" s="33"/>
+      <c r="I117" s="14">
+        <v>401</v>
+      </c>
       <c r="L117" s="5"/>
     </row>
-    <row r="118" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="118" spans="1:12" ht="20.65" thickBot="1">
       <c r="A118" s="34">
         <v>6</v>
       </c>
@@ -3945,10 +4099,12 @@
       <c r="H118" s="33">
         <v>2930.7765720000002</v>
       </c>
-      <c r="I118" s="33"/>
+      <c r="I118" s="14">
+        <v>401</v>
+      </c>
       <c r="L118" s="5"/>
     </row>
-    <row r="119" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="119" spans="1:12" ht="20.65" thickBot="1">
       <c r="A119" s="34">
         <v>6</v>
       </c>
@@ -3973,10 +4129,12 @@
       <c r="H119" s="33">
         <v>1634.5169000000001</v>
       </c>
-      <c r="I119" s="33"/>
+      <c r="I119" s="14">
+        <v>401</v>
+      </c>
       <c r="L119" s="5"/>
     </row>
-    <row r="120" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="120" spans="1:12" ht="20.65" thickBot="1">
       <c r="A120" s="34">
         <v>6</v>
       </c>
@@ -4001,10 +4159,12 @@
       <c r="H120" s="33">
         <v>2699.044245</v>
       </c>
-      <c r="I120" s="33"/>
+      <c r="I120" s="14">
+        <v>401</v>
+      </c>
       <c r="L120" s="5"/>
     </row>
-    <row r="121" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="121" spans="1:12" ht="20.65" thickBot="1">
       <c r="A121" s="34">
         <v>6</v>
       </c>
@@ -4029,10 +4189,12 @@
       <c r="H121" s="33">
         <v>2367.4099289999999</v>
       </c>
-      <c r="I121" s="33"/>
+      <c r="I121" s="14">
+        <v>401</v>
+      </c>
       <c r="L121" s="5"/>
     </row>
-    <row r="122" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="122" spans="1:12" ht="20.65" thickBot="1">
       <c r="A122" s="34">
         <v>6</v>
       </c>
@@ -4057,10 +4219,12 @@
       <c r="H122" s="33">
         <v>4761.7163840000003</v>
       </c>
-      <c r="I122" s="33"/>
+      <c r="I122" s="14">
+        <v>401</v>
+      </c>
       <c r="L122" s="5"/>
     </row>
-    <row r="123" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="123" spans="1:12" ht="20.65" thickBot="1">
       <c r="A123" s="34">
         <v>6</v>
       </c>
@@ -4085,10 +4249,12 @@
       <c r="H123" s="33">
         <v>5361.1084309999997</v>
       </c>
-      <c r="I123" s="33"/>
+      <c r="I123" s="14">
+        <v>401</v>
+      </c>
       <c r="L123" s="5"/>
     </row>
-    <row r="124" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="124" spans="1:12" ht="20.65" thickBot="1">
       <c r="A124" s="34">
         <v>6</v>
       </c>
@@ -4113,10 +4279,12 @@
       <c r="H124" s="33">
         <v>4696.9448110000003</v>
       </c>
-      <c r="I124" s="33"/>
+      <c r="I124" s="14">
+        <v>401</v>
+      </c>
       <c r="L124" s="5"/>
     </row>
-    <row r="125" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="125" spans="1:12" ht="20.65" thickBot="1">
       <c r="A125" s="34">
         <v>6</v>
       </c>
@@ -4141,10 +4309,12 @@
       <c r="H125" s="33">
         <v>5097.0499840000002</v>
       </c>
-      <c r="I125" s="33"/>
+      <c r="I125" s="14">
+        <v>401</v>
+      </c>
       <c r="L125" s="5"/>
     </row>
-    <row r="126" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="126" spans="1:12" ht="20.65" thickBot="1">
       <c r="A126" s="34">
         <v>6</v>
       </c>
@@ -4169,10 +4339,12 @@
       <c r="H126" s="33">
         <v>3302.9510100000002</v>
       </c>
-      <c r="I126" s="33"/>
+      <c r="I126" s="14">
+        <v>401</v>
+      </c>
       <c r="L126" s="5"/>
     </row>
-    <row r="127" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="127" spans="1:12" ht="20.65" thickBot="1">
       <c r="A127" s="34">
         <v>6</v>
       </c>
@@ -4197,10 +4369,12 @@
       <c r="H127" s="33">
         <v>4899.0757590000003</v>
       </c>
-      <c r="I127" s="33"/>
+      <c r="I127" s="14">
+        <v>401</v>
+      </c>
       <c r="L127" s="5"/>
     </row>
-    <row r="128" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="128" spans="1:12" ht="20.65" thickBot="1">
       <c r="A128" s="34">
         <v>6</v>
       </c>
@@ -4225,10 +4399,12 @@
       <c r="H128" s="33">
         <v>1509.806691</v>
       </c>
-      <c r="I128" s="33"/>
+      <c r="I128" s="14">
+        <v>401</v>
+      </c>
       <c r="L128" s="5"/>
     </row>
-    <row r="129" spans="1:13" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="129" spans="1:13" ht="20.65" thickBot="1">
       <c r="A129" s="34">
         <v>6</v>
       </c>
@@ -4253,10 +4429,12 @@
       <c r="H129" s="33">
         <v>14.89658092</v>
       </c>
-      <c r="I129" s="33"/>
+      <c r="I129" s="14">
+        <v>401</v>
+      </c>
       <c r="L129" s="5"/>
     </row>
-    <row r="130" spans="1:13" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="130" spans="1:13" ht="20.65" thickBot="1">
       <c r="A130" s="34">
         <v>6</v>
       </c>
@@ -4281,11 +4459,13 @@
       <c r="H130" s="33">
         <v>1378.712233</v>
       </c>
-      <c r="I130" s="33"/>
+      <c r="I130" s="14">
+        <v>401</v>
+      </c>
       <c r="L130" s="3"/>
       <c r="M130" s="3"/>
     </row>
-    <row r="131" spans="1:13" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="131" spans="1:13" ht="20.65" thickBot="1">
       <c r="A131" s="34">
         <v>6</v>
       </c>
@@ -4310,11 +4490,13 @@
       <c r="H131" s="33">
         <v>9889.18318</v>
       </c>
-      <c r="I131" s="33"/>
+      <c r="I131" s="14">
+        <v>401</v>
+      </c>
       <c r="L131" s="2"/>
       <c r="M131" s="3"/>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:13">
       <c r="A132" s="35">
         <v>6</v>
       </c>
@@ -4339,11 +4521,13 @@
       <c r="H132" s="33">
         <v>17.561656809999999</v>
       </c>
-      <c r="I132" s="33"/>
+      <c r="I132" s="14">
+        <v>401</v>
+      </c>
       <c r="L132" s="2"/>
       <c r="M132" s="3"/>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:13">
       <c r="A133" s="37">
         <v>7</v>
       </c>
@@ -4374,7 +4558,7 @@
       <c r="L133" s="2"/>
       <c r="M133" s="3"/>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:13">
       <c r="A134" s="34">
         <v>7</v>
       </c>
@@ -4399,11 +4583,13 @@
       <c r="H134" s="33">
         <v>21.604938270000002</v>
       </c>
-      <c r="I134" s="33"/>
+      <c r="I134" s="14">
+        <v>346</v>
+      </c>
       <c r="L134" s="2"/>
       <c r="M134" s="3"/>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:13">
       <c r="A135" s="34">
         <v>7</v>
       </c>
@@ -4428,11 +4614,13 @@
       <c r="H135" s="33">
         <v>367.28395060000003</v>
       </c>
-      <c r="I135" s="33"/>
+      <c r="I135" s="14">
+        <v>346</v>
+      </c>
       <c r="L135" s="2"/>
       <c r="M135" s="3"/>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:13">
       <c r="A136" s="34">
         <v>7</v>
       </c>
@@ -4457,11 +4645,13 @@
       <c r="H136" s="33">
         <v>1555.555556</v>
       </c>
-      <c r="I136" s="33"/>
+      <c r="I136" s="14">
+        <v>346</v>
+      </c>
       <c r="L136" s="2"/>
       <c r="M136" s="3"/>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:13">
       <c r="A137" s="34">
         <v>7</v>
       </c>
@@ -4486,11 +4676,13 @@
       <c r="H137" s="33">
         <v>2074.0740740000001</v>
       </c>
-      <c r="I137" s="33"/>
+      <c r="I137" s="14">
+        <v>346</v>
+      </c>
       <c r="L137" s="2"/>
       <c r="M137" s="3"/>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:13">
       <c r="A138" s="34">
         <v>7</v>
       </c>
@@ -4515,11 +4707,13 @@
       <c r="H138" s="33">
         <v>3132.7160490000001</v>
       </c>
-      <c r="I138" s="33"/>
+      <c r="I138" s="14">
+        <v>346</v>
+      </c>
       <c r="L138" s="2"/>
       <c r="M138" s="3"/>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:13">
       <c r="A139" s="34">
         <v>7</v>
       </c>
@@ -4544,11 +4738,13 @@
       <c r="H139" s="33">
         <v>3175.9259259999999</v>
       </c>
-      <c r="I139" s="33"/>
+      <c r="I139" s="14">
+        <v>346</v>
+      </c>
       <c r="L139" s="2"/>
       <c r="M139" s="3"/>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:13">
       <c r="A140" s="34">
         <v>7</v>
       </c>
@@ -4573,11 +4769,13 @@
       <c r="H140" s="33">
         <v>3391.9753089999999</v>
       </c>
-      <c r="I140" s="33"/>
+      <c r="I140" s="14">
+        <v>346</v>
+      </c>
       <c r="L140" s="2"/>
       <c r="M140" s="3"/>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:13">
       <c r="A141" s="34">
         <v>7</v>
       </c>
@@ -4602,10 +4800,12 @@
       <c r="H141" s="33">
         <v>4277.7777779999997</v>
       </c>
-      <c r="I141" s="33"/>
+      <c r="I141" s="14">
+        <v>346</v>
+      </c>
       <c r="L141" s="5"/>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:13">
       <c r="A142" s="34">
         <v>7</v>
       </c>
@@ -4630,10 +4830,12 @@
       <c r="H142" s="33">
         <v>4472.2222220000003</v>
       </c>
-      <c r="I142" s="33"/>
+      <c r="I142" s="14">
+        <v>346</v>
+      </c>
       <c r="L142" s="5"/>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:13">
       <c r="A143" s="34">
         <v>7</v>
       </c>
@@ -4658,10 +4860,12 @@
       <c r="H143" s="33">
         <v>4472.2222220000003</v>
       </c>
-      <c r="I143" s="33"/>
+      <c r="I143" s="14">
+        <v>346</v>
+      </c>
       <c r="L143" s="5"/>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:13">
       <c r="A144" s="34">
         <v>7</v>
       </c>
@@ -4686,10 +4890,12 @@
       <c r="H144" s="33">
         <v>4407.4074069999997</v>
       </c>
-      <c r="I144" s="33"/>
+      <c r="I144" s="14">
+        <v>346</v>
+      </c>
       <c r="L144" s="5"/>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:12">
       <c r="A145" s="34">
         <v>7</v>
       </c>
@@ -4714,10 +4920,12 @@
       <c r="H145" s="33">
         <v>3478.3950620000001</v>
       </c>
-      <c r="I145" s="33"/>
+      <c r="I145" s="14">
+        <v>346</v>
+      </c>
       <c r="L145" s="5"/>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:12">
       <c r="A146" s="34">
         <v>7</v>
       </c>
@@ -4742,10 +4950,12 @@
       <c r="H146" s="33">
         <v>3262.345679</v>
       </c>
-      <c r="I146" s="33"/>
+      <c r="I146" s="14">
+        <v>346</v>
+      </c>
       <c r="L146" s="5"/>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:12">
       <c r="A147" s="34">
         <v>7</v>
       </c>
@@ -4770,10 +4980,12 @@
       <c r="H147" s="33">
         <v>3089.5061730000002</v>
       </c>
-      <c r="I147" s="33"/>
+      <c r="I147" s="14">
+        <v>346</v>
+      </c>
       <c r="L147" s="5"/>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:12">
       <c r="A148" s="34">
         <v>7</v>
       </c>
@@ -4798,10 +5010,12 @@
       <c r="H148" s="33">
         <v>3024.691358</v>
       </c>
-      <c r="I148" s="33"/>
+      <c r="I148" s="14">
+        <v>346</v>
+      </c>
       <c r="L148" s="5"/>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:12">
       <c r="A149" s="34">
         <v>7</v>
       </c>
@@ -4826,10 +5040,12 @@
       <c r="H149" s="33">
         <v>2527.7777780000001</v>
       </c>
-      <c r="I149" s="33"/>
+      <c r="I149" s="14">
+        <v>346</v>
+      </c>
       <c r="L149" s="5"/>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:12">
       <c r="A150" s="34">
         <v>7</v>
       </c>
@@ -4854,10 +5070,12 @@
       <c r="H150" s="33">
         <v>1469.135802</v>
       </c>
-      <c r="I150" s="33"/>
+      <c r="I150" s="14">
+        <v>346</v>
+      </c>
       <c r="L150" s="5"/>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:12">
       <c r="A151" s="34">
         <v>7</v>
       </c>
@@ -4882,10 +5100,12 @@
       <c r="H151" s="33">
         <v>151.2345679</v>
       </c>
-      <c r="I151" s="33"/>
+      <c r="I151" s="14">
+        <v>346</v>
+      </c>
       <c r="L151" s="5"/>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:12">
       <c r="A152" s="34">
         <v>7</v>
       </c>
@@ -4910,10 +5130,12 @@
       <c r="H152" s="33">
         <v>280.86419749999999</v>
       </c>
-      <c r="I152" s="33"/>
+      <c r="I152" s="14">
+        <v>346</v>
+      </c>
       <c r="L152" s="5"/>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:12">
       <c r="A153" s="35">
         <v>7</v>
       </c>
@@ -4938,10 +5160,12 @@
       <c r="H153" s="33">
         <v>0</v>
       </c>
-      <c r="I153" s="33"/>
+      <c r="I153" s="14">
+        <v>346</v>
+      </c>
       <c r="L153" s="5"/>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:12">
       <c r="A154" s="37">
         <v>8</v>
       </c>
@@ -4975,7 +5199,7 @@
       <c r="K154" s="7"/>
       <c r="L154" s="5"/>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:12">
       <c r="A155" s="34">
         <v>8</v>
       </c>
@@ -5000,10 +5224,12 @@
       <c r="H155" s="33">
         <v>843.37349400000005</v>
       </c>
-      <c r="I155" s="33"/>
+      <c r="I155" s="14">
+        <v>136</v>
+      </c>
       <c r="L155" s="5"/>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:12">
       <c r="A156" s="34">
         <v>8</v>
       </c>
@@ -5028,10 +5254,12 @@
       <c r="H156" s="33">
         <v>6662.6506019999997</v>
       </c>
-      <c r="I156" s="33"/>
+      <c r="I156" s="14">
+        <v>136</v>
+      </c>
       <c r="L156" s="5"/>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:12">
       <c r="A157" s="34">
         <v>8</v>
       </c>
@@ -5056,10 +5284,12 @@
       <c r="H157" s="33">
         <v>168.67469879999999</v>
       </c>
-      <c r="I157" s="33"/>
+      <c r="I157" s="14">
+        <v>136</v>
+      </c>
       <c r="L157" s="5"/>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:12">
       <c r="A158" s="34">
         <v>8</v>
       </c>
@@ -5084,10 +5314,12 @@
       <c r="H158" s="33">
         <v>927.71084340000004</v>
       </c>
-      <c r="I158" s="33"/>
+      <c r="I158" s="14">
+        <v>136</v>
+      </c>
       <c r="L158" s="5"/>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:12">
       <c r="A159" s="34">
         <v>8</v>
       </c>
@@ -5112,10 +5344,12 @@
       <c r="H159" s="33">
         <v>801.20481930000005</v>
       </c>
-      <c r="I159" s="33"/>
+      <c r="I159" s="14">
+        <v>136</v>
+      </c>
       <c r="L159" s="5"/>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:12">
       <c r="A160" s="34">
         <v>8</v>
       </c>
@@ -5140,10 +5374,12 @@
       <c r="H160" s="33">
         <v>1644.578313</v>
       </c>
-      <c r="I160" s="33"/>
+      <c r="I160" s="14">
+        <v>136</v>
+      </c>
       <c r="L160" s="5"/>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:12">
       <c r="A161" s="34">
         <v>8</v>
       </c>
@@ -5168,10 +5404,12 @@
       <c r="H161" s="33">
         <v>1391.5662649999999</v>
       </c>
-      <c r="I161" s="33"/>
+      <c r="I161" s="14">
+        <v>136</v>
+      </c>
       <c r="L161" s="5"/>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:12">
       <c r="A162" s="34">
         <v>8</v>
       </c>
@@ -5196,10 +5434,12 @@
       <c r="H162" s="33">
         <v>1602.409639</v>
       </c>
-      <c r="I162" s="33"/>
+      <c r="I162" s="14">
+        <v>136</v>
+      </c>
       <c r="L162" s="5"/>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:12">
       <c r="A163" s="34">
         <v>8</v>
       </c>
@@ -5224,10 +5464,12 @@
       <c r="H163" s="33">
         <v>1855.421687</v>
       </c>
-      <c r="I163" s="33"/>
+      <c r="I163" s="14">
+        <v>136</v>
+      </c>
       <c r="L163" s="5"/>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:12">
       <c r="A164" s="34">
         <v>8</v>
       </c>
@@ -5252,10 +5494,12 @@
       <c r="H164" s="33">
         <v>1096.385542</v>
       </c>
-      <c r="I164" s="33"/>
+      <c r="I164" s="14">
+        <v>136</v>
+      </c>
       <c r="L164" s="5"/>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:12">
       <c r="A165" s="34">
         <v>8</v>
       </c>
@@ -5280,10 +5524,12 @@
       <c r="H165" s="33">
         <v>1012.048193</v>
       </c>
-      <c r="I165" s="33"/>
+      <c r="I165" s="14">
+        <v>136</v>
+      </c>
       <c r="L165" s="5"/>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:12">
       <c r="A166" s="34">
         <v>8</v>
       </c>
@@ -5308,10 +5554,12 @@
       <c r="H166" s="33">
         <v>1012.048193</v>
       </c>
-      <c r="I166" s="33"/>
+      <c r="I166" s="14">
+        <v>136</v>
+      </c>
       <c r="L166" s="5"/>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:12">
       <c r="A167" s="34">
         <v>8</v>
       </c>
@@ -5336,10 +5584,12 @@
       <c r="H167" s="33">
         <v>1012.048193</v>
       </c>
-      <c r="I167" s="33"/>
+      <c r="I167" s="14">
+        <v>136</v>
+      </c>
       <c r="L167" s="5"/>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:12">
       <c r="A168" s="34">
         <v>8</v>
       </c>
@@ -5364,10 +5614,12 @@
       <c r="H168" s="33">
         <v>590.36144579999996</v>
       </c>
-      <c r="I168" s="33"/>
+      <c r="I168" s="14">
+        <v>136</v>
+      </c>
       <c r="L168" s="5"/>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:12">
       <c r="A169" s="34">
         <v>8</v>
       </c>
@@ -5392,10 +5644,12 @@
       <c r="H169" s="33">
         <v>253.01204820000001</v>
       </c>
-      <c r="I169" s="33"/>
+      <c r="I169" s="14">
+        <v>136</v>
+      </c>
       <c r="L169" s="5"/>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:12">
       <c r="A170" s="34">
         <v>8</v>
       </c>
@@ -5420,10 +5674,12 @@
       <c r="H170" s="33">
         <v>674.69879519999995</v>
       </c>
-      <c r="I170" s="33"/>
+      <c r="I170" s="14">
+        <v>136</v>
+      </c>
       <c r="L170" s="5"/>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:12">
       <c r="A171" s="34">
         <v>8</v>
       </c>
@@ -5448,10 +5704,12 @@
       <c r="H171" s="33">
         <v>168.67469879999999</v>
       </c>
-      <c r="I171" s="33"/>
+      <c r="I171" s="14">
+        <v>136</v>
+      </c>
       <c r="L171" s="5"/>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:12">
       <c r="A172" s="34">
         <v>8</v>
       </c>
@@ -5476,10 +5734,12 @@
       <c r="H172" s="33">
         <v>126.5060241</v>
       </c>
-      <c r="I172" s="33"/>
+      <c r="I172" s="14">
+        <v>136</v>
+      </c>
       <c r="L172" s="5"/>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:12">
       <c r="A173" s="34">
         <v>8</v>
       </c>
@@ -5504,10 +5764,12 @@
       <c r="H173" s="33">
         <v>84.337349399999994</v>
       </c>
-      <c r="I173" s="33"/>
+      <c r="I173" s="14">
+        <v>136</v>
+      </c>
       <c r="L173" s="5"/>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:12">
       <c r="A174" s="34">
         <v>8</v>
       </c>
@@ -5532,10 +5794,12 @@
       <c r="H174" s="33">
         <v>0</v>
       </c>
-      <c r="I174" s="33"/>
+      <c r="I174" s="14">
+        <v>136</v>
+      </c>
       <c r="L174" s="5"/>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:12">
       <c r="A175" s="35">
         <v>8</v>
       </c>
@@ -5560,10 +5824,12 @@
       <c r="H175" s="33">
         <v>0</v>
       </c>
-      <c r="I175" s="33"/>
+      <c r="I175" s="14">
+        <v>136</v>
+      </c>
       <c r="L175" s="5"/>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:12">
       <c r="A176" s="37">
         <v>9</v>
       </c>
@@ -5597,7 +5863,7 @@
       <c r="K176" s="7"/>
       <c r="L176" s="5"/>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:12">
       <c r="A177" s="34">
         <v>9</v>
       </c>
@@ -5622,10 +5888,12 @@
       <c r="H177" s="33">
         <v>0</v>
       </c>
-      <c r="I177" s="33"/>
+      <c r="I177" s="14">
+        <v>57</v>
+      </c>
       <c r="L177" s="5"/>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:12">
       <c r="A178" s="34">
         <v>9</v>
       </c>
@@ -5650,10 +5918,12 @@
       <c r="H178" s="33">
         <v>0</v>
       </c>
-      <c r="I178" s="33"/>
+      <c r="I178" s="14">
+        <v>57</v>
+      </c>
       <c r="L178" s="5"/>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="179" spans="1:12">
       <c r="A179" s="34">
         <v>9</v>
       </c>
@@ -5678,10 +5948,12 @@
       <c r="H179" s="33">
         <v>44.943820219999999</v>
       </c>
-      <c r="I179" s="33"/>
+      <c r="I179" s="14">
+        <v>57</v>
+      </c>
       <c r="L179" s="5"/>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="180" spans="1:12">
       <c r="A180" s="34">
         <v>9</v>
       </c>
@@ -5706,10 +5978,12 @@
       <c r="H180" s="33">
         <v>152.80898880000001</v>
       </c>
-      <c r="I180" s="33"/>
+      <c r="I180" s="14">
+        <v>57</v>
+      </c>
       <c r="L180" s="5"/>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="181" spans="1:12">
       <c r="A181" s="34">
         <v>9</v>
       </c>
@@ -5734,10 +6008,12 @@
       <c r="H181" s="33">
         <v>53.93258427</v>
       </c>
-      <c r="I181" s="33"/>
+      <c r="I181" s="14">
+        <v>57</v>
+      </c>
       <c r="L181" s="5"/>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:12">
       <c r="A182" s="34">
         <v>9</v>
       </c>
@@ -5762,10 +6038,12 @@
       <c r="H182" s="33">
         <v>94.382022469999995</v>
       </c>
-      <c r="I182" s="33"/>
+      <c r="I182" s="14">
+        <v>57</v>
+      </c>
       <c r="L182" s="5"/>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:12">
       <c r="A183" s="34">
         <v>9</v>
       </c>
@@ -5790,10 +6068,12 @@
       <c r="H183" s="33">
         <v>49.438202250000003</v>
       </c>
-      <c r="I183" s="33"/>
+      <c r="I183" s="14">
+        <v>57</v>
+      </c>
       <c r="L183" s="5"/>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="184" spans="1:12">
       <c r="A184" s="34">
         <v>9</v>
       </c>
@@ -5818,10 +6098,12 @@
       <c r="H184" s="33">
         <v>89.887640450000006</v>
       </c>
-      <c r="I184" s="33"/>
+      <c r="I184" s="14">
+        <v>57</v>
+      </c>
       <c r="L184" s="5"/>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="185" spans="1:12">
       <c r="A185" s="34">
         <v>9</v>
       </c>
@@ -5846,10 +6128,12 @@
       <c r="H185" s="33">
         <v>98.876404489999999</v>
       </c>
-      <c r="I185" s="33"/>
+      <c r="I185" s="14">
+        <v>57</v>
+      </c>
       <c r="L185" s="5"/>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="186" spans="1:12">
       <c r="A186" s="34">
         <v>9</v>
       </c>
@@ -5874,10 +6158,12 @@
       <c r="H186" s="33">
         <v>404.49438199999997</v>
       </c>
-      <c r="I186" s="33"/>
+      <c r="I186" s="14">
+        <v>57</v>
+      </c>
       <c r="L186" s="5"/>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="187" spans="1:12">
       <c r="A187" s="34">
         <v>9</v>
       </c>
@@ -5902,10 +6188,12 @@
       <c r="H187" s="33">
         <v>444.9438202</v>
       </c>
-      <c r="I187" s="33"/>
+      <c r="I187" s="14">
+        <v>57</v>
+      </c>
       <c r="L187" s="5"/>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="188" spans="1:12">
       <c r="A188" s="34">
         <v>9</v>
       </c>
@@ -5930,10 +6218,12 @@
       <c r="H188" s="33">
         <v>804.49438199999997</v>
       </c>
-      <c r="I188" s="33"/>
+      <c r="I188" s="14">
+        <v>57</v>
+      </c>
       <c r="L188" s="5"/>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:12">
       <c r="A189" s="34">
         <v>9</v>
       </c>
@@ -5958,10 +6248,12 @@
       <c r="H189" s="33">
         <v>611.23595509999996</v>
       </c>
-      <c r="I189" s="33"/>
+      <c r="I189" s="14">
+        <v>57</v>
+      </c>
       <c r="L189" s="5"/>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="190" spans="1:12">
       <c r="A190" s="34">
         <v>9</v>
       </c>
@@ -5986,10 +6278,12 @@
       <c r="H190" s="33">
         <v>853.93258430000003</v>
       </c>
-      <c r="I190" s="33"/>
+      <c r="I190" s="14">
+        <v>57</v>
+      </c>
       <c r="L190" s="5"/>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:12">
       <c r="A191" s="34">
         <v>9</v>
       </c>
@@ -6014,10 +6308,12 @@
       <c r="H191" s="33">
         <v>840.44943820000003</v>
       </c>
-      <c r="I191" s="33"/>
+      <c r="I191" s="14">
+        <v>57</v>
+      </c>
       <c r="L191" s="5"/>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="192" spans="1:12">
       <c r="A192" s="34">
         <v>9</v>
       </c>
@@ -6042,10 +6338,12 @@
       <c r="H192" s="33">
         <v>1271.910112</v>
       </c>
-      <c r="I192" s="33"/>
+      <c r="I192" s="14">
+        <v>57</v>
+      </c>
       <c r="L192" s="5"/>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="193" spans="1:12">
       <c r="A193" s="34">
         <v>9</v>
       </c>
@@ -6070,10 +6368,12 @@
       <c r="H193" s="33">
         <v>975.28089890000001</v>
       </c>
-      <c r="I193" s="33"/>
+      <c r="I193" s="14">
+        <v>57</v>
+      </c>
       <c r="L193" s="5"/>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:12">
       <c r="A194" s="34">
         <v>9</v>
       </c>
@@ -6098,10 +6398,12 @@
       <c r="H194" s="33">
         <v>633.70786520000001</v>
       </c>
-      <c r="I194" s="33"/>
+      <c r="I194" s="14">
+        <v>57</v>
+      </c>
       <c r="L194" s="5"/>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:12">
       <c r="A195" s="34">
         <v>9</v>
       </c>
@@ -6126,10 +6428,12 @@
       <c r="H195" s="33">
         <v>759.55056179999997</v>
       </c>
-      <c r="I195" s="33"/>
+      <c r="I195" s="14">
+        <v>57</v>
+      </c>
       <c r="L195" s="5"/>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="196" spans="1:12">
       <c r="A196" s="34">
         <v>9</v>
       </c>
@@ -6154,10 +6458,12 @@
       <c r="H196" s="33">
         <v>350.56179780000002</v>
       </c>
-      <c r="I196" s="33"/>
+      <c r="I196" s="14">
+        <v>57</v>
+      </c>
       <c r="L196" s="5"/>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:12">
       <c r="A197" s="34">
         <v>9</v>
       </c>
@@ -6182,10 +6488,12 @@
       <c r="H197" s="33">
         <v>157.30337080000001</v>
       </c>
-      <c r="I197" s="33"/>
+      <c r="I197" s="14">
+        <v>57</v>
+      </c>
       <c r="L197" s="5"/>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="198" spans="1:12">
       <c r="A198" s="34">
         <v>9</v>
       </c>
@@ -6210,10 +6518,12 @@
       <c r="H198" s="33">
         <v>80.898876400000006</v>
       </c>
-      <c r="I198" s="33"/>
+      <c r="I198" s="14">
+        <v>57</v>
+      </c>
       <c r="L198" s="5"/>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:12">
       <c r="A199" s="34">
         <v>9</v>
       </c>
@@ -6238,10 +6548,12 @@
       <c r="H199" s="33">
         <v>0</v>
       </c>
-      <c r="I199" s="33"/>
+      <c r="I199" s="14">
+        <v>57</v>
+      </c>
       <c r="L199" s="5"/>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:12">
       <c r="A200" s="35">
         <v>9</v>
       </c>
@@ -6266,10 +6578,12 @@
       <c r="H200" s="33">
         <v>0</v>
       </c>
-      <c r="I200" s="33"/>
+      <c r="I200" s="14">
+        <v>57</v>
+      </c>
       <c r="L200" s="5"/>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:12">
       <c r="A201" s="37">
         <v>10</v>
       </c>
@@ -6299,7 +6613,7 @@
       </c>
       <c r="L201" s="5"/>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:12">
       <c r="A202" s="34">
         <v>10</v>
       </c>
@@ -6324,10 +6638,12 @@
       <c r="H202" s="33">
         <v>0</v>
       </c>
-      <c r="I202" s="33"/>
+      <c r="I202" s="14">
+        <v>38</v>
+      </c>
       <c r="L202" s="5"/>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="203" spans="1:12">
       <c r="A203" s="34">
         <v>10</v>
       </c>
@@ -6352,10 +6668,12 @@
       <c r="H203" s="33">
         <v>36.011080329999999</v>
       </c>
-      <c r="I203" s="33"/>
+      <c r="I203" s="14">
+        <v>38</v>
+      </c>
       <c r="L203" s="5"/>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:12">
       <c r="A204" s="34">
         <v>10</v>
       </c>
@@ -6380,10 +6698,12 @@
       <c r="H204" s="33">
         <v>121.8836565</v>
       </c>
-      <c r="I204" s="33"/>
+      <c r="I204" s="14">
+        <v>38</v>
+      </c>
       <c r="L204" s="5"/>
     </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:12">
       <c r="A205" s="34">
         <v>10</v>
       </c>
@@ -6408,10 +6728,12 @@
       <c r="H205" s="33">
         <v>49.861495840000003</v>
       </c>
-      <c r="I205" s="33"/>
+      <c r="I205" s="14">
+        <v>38</v>
+      </c>
       <c r="L205" s="5"/>
     </row>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="206" spans="1:12">
       <c r="A206" s="34">
         <v>10</v>
       </c>
@@ -6436,10 +6758,12 @@
       <c r="H206" s="33">
         <v>545.70637120000004</v>
       </c>
-      <c r="I206" s="33"/>
+      <c r="I206" s="14">
+        <v>38</v>
+      </c>
       <c r="L206" s="5"/>
     </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:12">
       <c r="A207" s="34">
         <v>10</v>
       </c>
@@ -6464,10 +6788,12 @@
       <c r="H207" s="33">
         <v>80.33240997</v>
       </c>
-      <c r="I207" s="33"/>
+      <c r="I207" s="14">
+        <v>38</v>
+      </c>
       <c r="L207" s="5"/>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="208" spans="1:12">
       <c r="A208" s="34">
         <v>10</v>
       </c>
@@ -6492,10 +6818,12 @@
       <c r="H208" s="33">
         <v>282.54847649999999</v>
       </c>
-      <c r="I208" s="33"/>
+      <c r="I208" s="14">
+        <v>38</v>
+      </c>
       <c r="L208" s="5"/>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:12">
       <c r="A209" s="34">
         <v>10</v>
       </c>
@@ -6520,10 +6848,12 @@
       <c r="H209" s="33">
         <v>235.45706369999999</v>
       </c>
-      <c r="I209" s="33"/>
+      <c r="I209" s="14">
+        <v>38</v>
+      </c>
       <c r="L209" s="5"/>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:12">
       <c r="A210" s="34">
         <v>10</v>
       </c>
@@ -6548,10 +6878,12 @@
       <c r="H210" s="33">
         <v>432.13296400000002</v>
       </c>
-      <c r="I210" s="33"/>
+      <c r="I210" s="14">
+        <v>38</v>
+      </c>
       <c r="L210" s="5"/>
     </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:12">
       <c r="A211" s="34">
         <v>10</v>
       </c>
@@ -6576,10 +6908,12 @@
       <c r="H211" s="33">
         <v>614.95844880000004</v>
       </c>
-      <c r="I211" s="33"/>
+      <c r="I211" s="14">
+        <v>38</v>
+      </c>
       <c r="L211" s="5"/>
     </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="212" spans="1:12">
       <c r="A212" s="34">
         <v>10</v>
       </c>
@@ -6604,10 +6938,12 @@
       <c r="H212" s="33">
         <v>554.01662050000004</v>
       </c>
-      <c r="I212" s="33"/>
+      <c r="I212" s="14">
+        <v>38</v>
+      </c>
       <c r="L212" s="5"/>
     </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="213" spans="1:12">
       <c r="A213" s="34">
         <v>10</v>
       </c>
@@ -6632,10 +6968,12 @@
       <c r="H213" s="33">
         <v>944.59833800000001</v>
       </c>
-      <c r="I213" s="33"/>
+      <c r="I213" s="14">
+        <v>38</v>
+      </c>
       <c r="L213" s="5"/>
     </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:12">
       <c r="A214" s="34">
         <v>10</v>
       </c>
@@ -6660,10 +6998,12 @@
       <c r="H214" s="33">
         <v>739.61218840000004</v>
       </c>
-      <c r="I214" s="33"/>
+      <c r="I214" s="14">
+        <v>38</v>
+      </c>
       <c r="L214" s="5"/>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:12">
       <c r="A215" s="34">
         <v>10</v>
       </c>
@@ -6688,10 +7028,12 @@
       <c r="H215" s="33">
         <v>645.4293629</v>
       </c>
-      <c r="I215" s="33"/>
+      <c r="I215" s="14">
+        <v>38</v>
+      </c>
       <c r="L215" s="5"/>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="216" spans="1:12">
       <c r="A216" s="34">
         <v>10</v>
       </c>
@@ -6716,10 +7058,12 @@
       <c r="H216" s="33">
         <v>340.7202216</v>
       </c>
-      <c r="I216" s="33"/>
+      <c r="I216" s="14">
+        <v>38</v>
+      </c>
       <c r="L216" s="5"/>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:12">
       <c r="A217" s="34">
         <v>10</v>
       </c>
@@ -6744,10 +7088,12 @@
       <c r="H217" s="33">
         <v>116.3434903</v>
       </c>
-      <c r="I217" s="33"/>
+      <c r="I217" s="14">
+        <v>38</v>
+      </c>
       <c r="L217" s="5"/>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:12">
       <c r="A218" s="34">
         <v>10</v>
       </c>
@@ -6772,10 +7118,12 @@
       <c r="H218" s="33">
         <v>0</v>
       </c>
-      <c r="I218" s="33"/>
+      <c r="I218" s="14">
+        <v>38</v>
+      </c>
       <c r="L218" s="5"/>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:12">
       <c r="A219" s="34">
         <v>10</v>
       </c>
@@ -6800,10 +7148,12 @@
       <c r="H219" s="33">
         <v>30.470914130000001</v>
       </c>
-      <c r="I219" s="33"/>
+      <c r="I219" s="14">
+        <v>38</v>
+      </c>
       <c r="L219" s="5"/>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:12">
       <c r="A220" s="34">
         <v>10</v>
       </c>
@@ -6828,10 +7178,12 @@
       <c r="H220" s="33">
         <v>2.7700831020000001</v>
       </c>
-      <c r="I220" s="33"/>
+      <c r="I220" s="14">
+        <v>38</v>
+      </c>
       <c r="L220" s="5"/>
     </row>
-    <row r="221" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="221" spans="1:12" ht="20.65" thickBot="1">
       <c r="A221" s="39">
         <v>10</v>
       </c>
@@ -6856,10 +7208,12 @@
       <c r="H221" s="33">
         <v>0</v>
       </c>
-      <c r="I221" s="33"/>
+      <c r="I221" s="14">
+        <v>38</v>
+      </c>
       <c r="L221" s="5"/>
     </row>
-    <row r="222" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="222" spans="1:12" ht="20.65" thickBot="1">
       <c r="A222" s="41">
         <v>11</v>
       </c>
@@ -6889,7 +7243,7 @@
       </c>
       <c r="L222" s="5"/>
     </row>
-    <row r="223" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="223" spans="1:12" ht="20.65" thickBot="1">
       <c r="A223" s="42">
         <v>11</v>
       </c>
@@ -6914,10 +7268,12 @@
       <c r="H223" s="33">
         <v>94.095940959999993</v>
       </c>
-      <c r="I223" s="33"/>
+      <c r="I223" s="14">
+        <v>60</v>
+      </c>
       <c r="L223" s="5"/>
     </row>
-    <row r="224" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="224" spans="1:12" ht="20.65" thickBot="1">
       <c r="A224" s="42">
         <v>11</v>
       </c>
@@ -6942,10 +7298,12 @@
       <c r="H224" s="33">
         <v>287.82287819999999</v>
       </c>
-      <c r="I224" s="33"/>
+      <c r="I224" s="14">
+        <v>60</v>
+      </c>
       <c r="L224" s="5"/>
     </row>
-    <row r="225" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="225" spans="1:12" ht="20.65" thickBot="1">
       <c r="A225" s="42">
         <v>11</v>
       </c>
@@ -6970,10 +7328,12 @@
       <c r="H225" s="33">
         <v>426.19926199999998</v>
       </c>
-      <c r="I225" s="33"/>
+      <c r="I225" s="14">
+        <v>60</v>
+      </c>
       <c r="L225" s="5"/>
     </row>
-    <row r="226" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="226" spans="1:12" ht="20.65" thickBot="1">
       <c r="A226" s="42">
         <v>11</v>
       </c>
@@ -6998,10 +7358,12 @@
       <c r="H226" s="33">
         <v>774.90774910000005</v>
       </c>
-      <c r="I226" s="33"/>
+      <c r="I226" s="14">
+        <v>60</v>
+      </c>
       <c r="L226" s="5"/>
     </row>
-    <row r="227" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="227" spans="1:12" ht="20.65" thickBot="1">
       <c r="A227" s="42">
         <v>11</v>
       </c>
@@ -7026,10 +7388,12 @@
       <c r="H227" s="33">
         <v>869.00369000000001</v>
       </c>
-      <c r="I227" s="33"/>
+      <c r="I227" s="14">
+        <v>60</v>
+      </c>
       <c r="L227" s="5"/>
     </row>
-    <row r="228" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="228" spans="1:12" ht="20.65" thickBot="1">
       <c r="A228" s="42">
         <v>11</v>
       </c>
@@ -7054,10 +7418,12 @@
       <c r="H228" s="33">
         <v>918.81918819999999</v>
       </c>
-      <c r="I228" s="33"/>
+      <c r="I228" s="14">
+        <v>60</v>
+      </c>
       <c r="L228" s="5"/>
     </row>
-    <row r="229" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="229" spans="1:12" ht="20.65" thickBot="1">
       <c r="A229" s="42">
         <v>11</v>
       </c>
@@ -7082,10 +7448,12 @@
       <c r="H229" s="33">
         <v>891.14391139999998</v>
       </c>
-      <c r="I229" s="33"/>
+      <c r="I229" s="14">
+        <v>60</v>
+      </c>
       <c r="L229" s="5"/>
     </row>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="230" spans="1:12">
       <c r="A230" s="43">
         <v>11</v>
       </c>
@@ -7110,10 +7478,12 @@
       <c r="H230" s="33">
         <v>337.63837640000003</v>
       </c>
-      <c r="I230" s="33"/>
+      <c r="I230" s="14">
+        <v>60</v>
+      </c>
       <c r="L230" s="5"/>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="231" spans="1:12">
       <c r="A231" s="44">
         <v>12</v>
       </c>
@@ -7143,7 +7513,7 @@
       </c>
       <c r="L231" s="5"/>
     </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="232" spans="1:12">
       <c r="A232" s="42">
         <v>12</v>
       </c>
@@ -7168,10 +7538,12 @@
       <c r="H232" s="33">
         <v>94.095940959999993</v>
       </c>
-      <c r="I232" s="33"/>
+      <c r="I232" s="14">
+        <v>69</v>
+      </c>
       <c r="L232" s="5"/>
     </row>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="233" spans="1:12">
       <c r="A233" s="42">
         <v>12</v>
       </c>
@@ -7196,10 +7568,12 @@
       <c r="H233" s="33">
         <v>99.63099631</v>
       </c>
-      <c r="I233" s="33"/>
+      <c r="I233" s="14">
+        <v>69</v>
+      </c>
       <c r="L233" s="5"/>
     </row>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="234" spans="1:12">
       <c r="A234" s="42">
         <v>12</v>
       </c>
@@ -7224,10 +7598,12 @@
       <c r="H234" s="33">
         <v>487.08487079999998</v>
       </c>
-      <c r="I234" s="33"/>
+      <c r="I234" s="14">
+        <v>69</v>
+      </c>
       <c r="L234" s="5"/>
     </row>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="235" spans="1:12">
       <c r="A235" s="42">
         <v>12</v>
       </c>
@@ -7252,10 +7628,12 @@
       <c r="H235" s="33">
         <v>570.11070110000003</v>
       </c>
-      <c r="I235" s="33"/>
+      <c r="I235" s="14">
+        <v>69</v>
+      </c>
       <c r="L235" s="5"/>
     </row>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="236" spans="1:12">
       <c r="A236" s="42">
         <v>12</v>
       </c>
@@ -7280,10 +7658,12 @@
       <c r="H236" s="33">
         <v>846.86346860000003</v>
       </c>
-      <c r="I236" s="33"/>
+      <c r="I236" s="14">
+        <v>69</v>
+      </c>
       <c r="L236" s="5"/>
     </row>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="237" spans="1:12">
       <c r="A237" s="42">
         <v>12</v>
       </c>
@@ -7308,10 +7688,12 @@
       <c r="H237" s="33">
         <v>869.00369000000001</v>
       </c>
-      <c r="I237" s="33"/>
+      <c r="I237" s="14">
+        <v>69</v>
+      </c>
       <c r="L237" s="5"/>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="238" spans="1:12">
       <c r="A238" s="42">
         <v>12</v>
       </c>
@@ -7336,10 +7718,12 @@
       <c r="H238" s="33">
         <v>1173.431734</v>
       </c>
-      <c r="I238" s="33"/>
+      <c r="I238" s="14">
+        <v>69</v>
+      </c>
       <c r="L238" s="5"/>
     </row>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="239" spans="1:12">
       <c r="A239" s="42">
         <v>12</v>
       </c>
@@ -7364,10 +7748,12 @@
       <c r="H239" s="33">
         <v>852.39852399999995</v>
       </c>
-      <c r="I239" s="33"/>
+      <c r="I239" s="14">
+        <v>69</v>
+      </c>
       <c r="L239" s="5"/>
     </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="240" spans="1:12">
       <c r="A240" s="42">
         <v>12</v>
       </c>
@@ -7392,10 +7778,12 @@
       <c r="H240" s="33">
         <v>387.45387449999998</v>
       </c>
-      <c r="I240" s="33"/>
+      <c r="I240" s="14">
+        <v>69</v>
+      </c>
       <c r="L240" s="5"/>
     </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="241" spans="1:12">
       <c r="A241" s="43">
         <v>12</v>
       </c>
@@ -7420,10 +7808,12 @@
       <c r="H241" s="33">
         <v>343.17343169999998</v>
       </c>
-      <c r="I241" s="33"/>
+      <c r="I241" s="14">
+        <v>69</v>
+      </c>
       <c r="L241" s="5"/>
     </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="242" spans="1:12">
       <c r="A242" s="44">
         <v>13</v>
       </c>
@@ -7452,7 +7842,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="243" spans="1:12">
       <c r="A243" s="42">
         <v>13</v>
       </c>
@@ -7477,9 +7867,11 @@
       <c r="H243" s="26">
         <v>94.095940959409702</v>
       </c>
-      <c r="I243" s="26"/>
-    </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I243" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="244" spans="1:12">
       <c r="A244" s="42">
         <v>13</v>
       </c>
@@ -7504,9 +7896,11 @@
       <c r="H244" s="26">
         <v>94.095940959409702</v>
       </c>
-      <c r="I244" s="26"/>
-    </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I244" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="245" spans="1:12">
       <c r="A245" s="42">
         <v>13</v>
       </c>
@@ -7531,9 +7925,11 @@
       <c r="H245" s="26">
         <v>370.84870848708402</v>
       </c>
-      <c r="I245" s="26"/>
-    </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I245" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="246" spans="1:12">
       <c r="A246" s="42">
         <v>13</v>
       </c>
@@ -7558,9 +7954,11 @@
       <c r="H246" s="26">
         <v>442.80442804427997</v>
       </c>
-      <c r="I246" s="26"/>
-    </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I246" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="247" spans="1:12">
       <c r="A247" s="42">
         <v>13</v>
       </c>
@@ -7585,9 +7983,11 @@
       <c r="H247" s="26">
         <v>697.41697416974102</v>
       </c>
-      <c r="I247" s="26"/>
-    </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I247" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="248" spans="1:12">
       <c r="A248" s="42">
         <v>13</v>
       </c>
@@ -7612,9 +8012,11 @@
       <c r="H248" s="26">
         <v>990.77490774907699</v>
       </c>
-      <c r="I248" s="26"/>
-    </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I248" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="249" spans="1:12">
       <c r="A249" s="42">
         <v>13</v>
       </c>
@@ -7639,9 +8041,11 @@
       <c r="H249" s="26">
         <v>869.00369003690003</v>
       </c>
-      <c r="I249" s="26"/>
-    </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="I249" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="250" spans="1:12">
       <c r="A250" s="42">
         <v>13</v>
       </c>
@@ -7666,9 +8070,11 @@
       <c r="H250" s="26">
         <v>536.90036900369</v>
       </c>
-      <c r="I250" s="26"/>
-    </row>
-    <row r="251" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="I250" s="14">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="251" spans="1:12" ht="20.65" thickBot="1">
       <c r="A251" s="48">
         <v>13</v>
       </c>
@@ -7693,7 +8099,9 @@
       <c r="H251" s="26">
         <v>420.66420664206601</v>
       </c>
-      <c r="I251" s="26"/>
+      <c r="I251" s="14">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -7704,14 +8112,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="109.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.26953125" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="109.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15.4">
       <c r="A1" s="10" t="s">
         <v>3</v>
       </c>
@@ -7722,7 +8130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15.4">
       <c r="A2" s="11" t="s">
         <v>30</v>
       </c>
@@ -7733,7 +8141,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="15.4">
       <c r="A3" s="6" t="s">
         <v>31</v>
       </c>
@@ -7744,7 +8152,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="15.4">
       <c r="A4" s="6" t="s">
         <v>32</v>
       </c>
@@ -7755,7 +8163,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="15.4">
       <c r="A5" s="6" t="s">
         <v>43</v>
       </c>
@@ -7766,42 +8174,42 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="15.4">
       <c r="A6" s="6">
         <v>5</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
     </row>
-    <row r="7" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="15.4">
       <c r="A7" s="6">
         <v>6</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
     </row>
-    <row r="8" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="15.4">
       <c r="A8" s="6">
         <v>7</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
     </row>
-    <row r="9" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="15.4">
       <c r="A9" s="6">
         <v>8</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
     </row>
-    <row r="10" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="15.4">
       <c r="A10" s="6">
         <v>9</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="15.4">
       <c r="A11" s="6">
         <v>10</v>
       </c>

</xml_diff>